<commit_message>
Update mobidam schema, new dropdown value, info text
</commit_message>
<xml_diff>
--- a/ckanext/lhm/schemas/template_master.xlsx
+++ b/ckanext/lhm/schemas/template_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\home\mb\p2\ckanext-lhm\ckanext\lhm\schemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{886DE068-3F1A-460B-9707-8F09C8425FD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4042D2DB-E3BC-4A36-8A81-E967F2CA0174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Datenverzeichnis" sheetId="17" r:id="rId2"/>
     <sheet name="Katalogwerte" sheetId="18" r:id="rId3"/>
     <sheet name="Dienste und Dokumente" sheetId="19" r:id="rId4"/>
-    <sheet name="Wertelisten" sheetId="16" r:id="rId5"/>
+    <sheet name="Wertelisten" sheetId="16" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Metadaten!$A$1:$K$52</definedName>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="274">
   <si>
     <t>nein</t>
   </si>
@@ -879,6 +879,9 @@
   </si>
   <si>
     <t>HANDLUNGSRAEUME</t>
+  </si>
+  <si>
+    <t>Kontinuierlich</t>
   </si>
 </sst>
 </file>
@@ -2300,7 +2303,7 @@
         <v>243</v>
       </c>
       <c r="X3" s="1" t="s">
-        <v>142</v>
+        <v>273</v>
       </c>
       <c r="Y3" s="1" t="s">
         <v>268</v>
@@ -2368,7 +2371,7 @@
         <v>244</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Y4" s="1" t="s">
         <v>238</v>
@@ -2415,7 +2418,7 @@
         <v>245</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -2459,7 +2462,7 @@
         <v>246</v>
       </c>
       <c r="X6" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -2497,7 +2500,7 @@
         <v>247</v>
       </c>
       <c r="X7" s="1" t="s">
-        <v>104</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -2535,7 +2538,7 @@
         <v>248</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>260</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -2561,7 +2564,7 @@
         <v>249</v>
       </c>
       <c r="X9" s="1" t="s">
-        <v>240</v>
+        <v>260</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -2588,7 +2591,7 @@
         <v>250</v>
       </c>
       <c r="X10" s="1" t="s">
-        <v>261</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -2615,7 +2618,7 @@
         <v>251</v>
       </c>
       <c r="X11" s="1" t="s">
-        <v>105</v>
+        <v>261</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -2638,6 +2641,9 @@
       <c r="W12" s="2" t="s">
         <v>252</v>
       </c>
+      <c r="X12" s="1" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="13" spans="1:25">
       <c r="A13" s="1" t="s">
@@ -2865,7 +2871,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="XQ0ScWYg5BozhXTL3qD7Ja8vGQVkbfQ5TFCSSURIC86Jv4/h1sqsnzQtrCN2jIc/JaLOX4yoW3a7XLWJ6XSQpA==" saltValue="4n/cAA+cyycyOEXksfwb5A==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated schema mobidam, enable additional value for data dictionary format
</commit_message>
<xml_diff>
--- a/ckanext/lhm/schemas/template_master.xlsx
+++ b/ckanext/lhm/schemas/template_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\home\mb\p2\ckanext-lhm\ckanext\lhm\schemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A48E7AD-2F1F-43C2-A7D8-9CFD81F8EE7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE1CF971-7B3C-452D-A909-A7303BF5AF21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="275">
   <si>
     <t>nein</t>
   </si>
@@ -882,6 +882,9 @@
   </si>
   <si>
     <t>1.3.7.</t>
+  </si>
+  <si>
+    <t>NCLOB</t>
   </si>
 </sst>
 </file>
@@ -2659,6 +2662,9 @@
       <c r="R13" s="1" t="s">
         <v>263</v>
       </c>
+      <c r="U13" s="1" t="s">
+        <v>274</v>
+      </c>
       <c r="W13" s="2" t="s">
         <v>253</v>
       </c>
@@ -2871,7 +2877,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="XQ0ScWYg5BozhXTL3qD7Ja8vGQVkbfQ5TFCSSURIC86Jv4/h1sqsnzQtrCN2jIc/JaLOX4yoW3a7XLWJ6XSQpA==" saltValue="4n/cAA+cyycyOEXksfwb5A==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="Oh/ECc0vO+/uxnQkqvwgpsVffqZrLtev3CiwusMhBT+YP46xQygVx1/iwcUq78rOdi5nLLBYbTrjgEKig0lf0g==" saltValue="SGrbqBkN6UmHt7N2wYHrzw==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>